<commit_message>
TC26_POM_Loginmercury modified with excel data driven test cas, Locator file added new signoff locator,LoginKeyword file modified,updat sheet2 in logindata excel file
</commit_message>
<xml_diff>
--- a/TestData/LoginData.xlsx
+++ b/TestData/LoginData.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\PycharmProjects\robotframework\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3A22E47-9126-4886-A6EE-D651963BAB94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CBF00A0-1397-424A-ABD1-E675B190D1B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{B8496DF7-5763-4752-ACE5-A8444D8DD572}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{B8496DF7-5763-4752-ACE5-A8444D8DD572}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="11">
   <si>
     <t>${username}</t>
   </si>
@@ -57,6 +58,18 @@
   </si>
   <si>
     <t>adm123@yourstore.com</t>
+  </si>
+  <si>
+    <t>admin1</t>
+  </si>
+  <si>
+    <t>admin2</t>
+  </si>
+  <si>
+    <t>kr</t>
+  </si>
+  <si>
+    <t>abcd</t>
   </si>
 </sst>
 </file>
@@ -518,4 +531,66 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId4"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6104C5B-B8FC-4F54-BC71-0879E24E97E3}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.28515625" customWidth="1"/>
+    <col min="2" max="2" width="17.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
TestCaseSuite_init with Feature1 and feature2 files, __init__.robot file,TC26_pom_LoginMercury1 modified file
</commit_message>
<xml_diff>
--- a/TestData/LoginData.xlsx
+++ b/TestData/LoginData.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\PycharmProjects\robotframework\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CBF00A0-1397-424A-ABD1-E675B190D1B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9987021A-0B1D-4D32-A9C8-AFEDBEFD5672}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{B8496DF7-5763-4752-ACE5-A8444D8DD572}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{B8496DF7-5763-4752-ACE5-A8444D8DD572}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Login" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="13">
   <si>
     <t>${username}</t>
   </si>
@@ -70,6 +71,12 @@
   </si>
   <si>
     <t>abcd</t>
+  </si>
+  <si>
+    <t>username</t>
+  </si>
+  <si>
+    <t>password</t>
   </si>
 </sst>
 </file>
@@ -593,4 +600,34 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C79CF3BA-4C92-4C69-BEF8-B8A50AB30874}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
ReadExcel_TC, utils file,Excel_keywords.robot file
</commit_message>
<xml_diff>
--- a/TestData/LoginData.xlsx
+++ b/TestData/LoginData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\PycharmProjects\robotframework\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9987021A-0B1D-4D32-A9C8-AFEDBEFD5672}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0565659F-A66F-470E-8A68-BB99A9FF601C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{B8496DF7-5763-4752-ACE5-A8444D8DD572}"/>
+    <workbookView xWindow="1845" yWindow="1395" windowWidth="12960" windowHeight="8955" activeTab="2" xr2:uid="{B8496DF7-5763-4752-ACE5-A8444D8DD572}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="14">
   <si>
     <t>${username}</t>
   </si>
@@ -77,6 +77,9 @@
   </si>
   <si>
     <t>password</t>
+  </si>
+  <si>
+    <t>admin12pwd</t>
   </si>
 </sst>
 </file>
@@ -624,7 +627,7 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>